<commit_message>
Regenerated ref reports to reflect change
</commit_message>
<xml_diff>
--- a/tests/traces/h100/Falconsai_nsfw_image_detection__1016002_perf_report.xlsx
+++ b/tests/traces/h100/Falconsai_nsfw_image_detection__1016002_perf_report.xlsx
@@ -868,7 +868,7 @@
       </c>
       <c r="AA2" t="inlineStr">
         <is>
-          <t>[{'name': 'void at::native::(anonymous namespace)::vectorized_layer_norm_kernel&lt;c10::BFloat16, float&gt;(int, float, c10::BFloat16 const*, c10::BFloat16 const*, c10::BFloat16 const*, float*, float*, c10::BFloat16*)', 'stream': 7, 'count': 25, 'total_duration_us': np.float64(111.20100000000001), 'mean_duration_us': np.float64(4.448040000000001), 'median_duration_us': np.float64(4.448), 'std_dev_duration_us': np.float64(0.10934037863479323), 'min_duration_us': np.float64(4.256), 'max_duration_us': np.float64(4.64)}]</t>
+          <t>[{'name': 'void at::native::(anonymous namespace)::vectorized_layer_norm_kernel&lt;c10::BFloat16, float&gt;(int, float, c10::BFloat16 const*, c10::BFloat16 const*, c10::BFloat16 const*, float*, float*, c10::BFloat16*)', 'stream': 7, 'gpu_op_uid': 4048, 'count': 25, 'total_duration_us': np.float64(111.20100000000001), 'mean_duration_us': np.float64(4.448040000000001), 'median_duration_us': np.float64(4.448), 'std_dev_duration_us': np.float64(0.10934037863479323), 'min_duration_us': np.float64(4.256), 'max_duration_us': np.float64(4.64)}]</t>
         </is>
       </c>
       <c r="AB2" t="inlineStr">
@@ -1024,7 +1024,7 @@
       </c>
       <c r="AA3" t="inlineStr">
         <is>
-          <t>[{'name': 'void at::native::(anonymous namespace)::vectorized_layer_norm_kernel&lt;c10::BFloat16, float&gt;(int, float, c10::BFloat16 const*, c10::BFloat16 const*, c10::BFloat16 const*, float*, float*, c10::BFloat16*)', 'stream': 7, 'count': 25, 'total_duration_us': np.float64(111.20100000000001), 'mean_duration_us': np.float64(4.448040000000001), 'median_duration_us': np.float64(4.448), 'std_dev_duration_us': np.float64(0.10934037863479323), 'min_duration_us': np.float64(4.256), 'max_duration_us': np.float64(4.64)}]</t>
+          <t>[{'name': 'void at::native::(anonymous namespace)::vectorized_layer_norm_kernel&lt;c10::BFloat16, float&gt;(int, float, c10::BFloat16 const*, c10::BFloat16 const*, c10::BFloat16 const*, float*, float*, c10::BFloat16*)', 'stream': 7, 'gpu_op_uid': 4048, 'count': 25, 'total_duration_us': np.float64(111.20100000000001), 'mean_duration_us': np.float64(4.448040000000001), 'median_duration_us': np.float64(4.448), 'std_dev_duration_us': np.float64(0.10934037863479323), 'min_duration_us': np.float64(4.256), 'max_duration_us': np.float64(4.64)}]</t>
         </is>
       </c>
       <c r="AB3" t="inlineStr">
@@ -5380,7 +5380,7 @@
       </c>
       <c r="AL2" t="inlineStr">
         <is>
-          <t>[{'name': 'void cutlass::Kernel2&lt;cutlass_80_tensorop_bf16_s16816gemm_relu_bf16_128x64_64x6_tn_align8&gt;(cutlass_80_tensorop_bf16_s16816gemm_relu_bf16_128x64_64x6_tn_align8::Params)', 'stream': 7, 'count': 48, 'total_duration_us': np.float64(399.136), 'mean_duration_us': np.float64(8.315333333333333), 'median_duration_us': np.float64(8.256), 'std_dev_duration_us': np.float64(0.13305517861231703), 'min_duration_us': np.float64(8.128), 'max_duration_us': np.float64(8.64)}]</t>
+          <t>[{'name': 'void cutlass::Kernel2&lt;cutlass_80_tensorop_bf16_s16816gemm_relu_bf16_128x64_64x6_tn_align8&gt;(cutlass_80_tensorop_bf16_s16816gemm_relu_bf16_128x64_64x6_tn_align8::Params)', 'stream': 7, 'gpu_op_uid': 4056, 'count': 48, 'total_duration_us': np.float64(399.136), 'mean_duration_us': np.float64(8.315333333333333), 'median_duration_us': np.float64(8.256), 'std_dev_duration_us': np.float64(0.13305517861231703), 'min_duration_us': np.float64(8.128), 'max_duration_us': np.float64(8.64)}]</t>
         </is>
       </c>
       <c r="AM2" t="inlineStr">
@@ -5537,7 +5537,7 @@
       </c>
       <c r="AL3" t="inlineStr">
         <is>
-          <t>[{'name': 'sm90_xmma_gemm_bf16bf16_bf16f32_f32_tn_n_tilesize128x128x64_warpgroupsize1x1x1_execute_segment_k_off_kernel__5x_cublas', 'stream': 7, 'count': 12, 'total_duration_us': np.float64(166.59), 'mean_duration_us': np.float64(13.8825), 'median_duration_us': np.float64(13.8875), 'std_dev_duration_us': np.float64(0.10183278777813505), 'min_duration_us': np.float64(13.76), 'max_duration_us': np.float64(14.176)}]</t>
+          <t>[{'name': 'sm90_xmma_gemm_bf16bf16_bf16f32_f32_tn_n_tilesize128x128x64_warpgroupsize1x1x1_execute_segment_k_off_kernel__5x_cublas', 'stream': 7, 'gpu_op_uid': 4108, 'count': 12, 'total_duration_us': np.float64(166.59), 'mean_duration_us': np.float64(13.8825), 'median_duration_us': np.float64(13.8875), 'std_dev_duration_us': np.float64(0.10183278777813505), 'min_duration_us': np.float64(13.76), 'max_duration_us': np.float64(14.176)}]</t>
         </is>
       </c>
       <c r="AM3" t="inlineStr">
@@ -5694,7 +5694,7 @@
       </c>
       <c r="AL4" t="inlineStr">
         <is>
-          <t>[{'name': 'sm90_xmma_gemm_bf16bf16_bf16f32_f32_tn_n_tilesize128x64x64_warpgroupsize1x1x1_execute_segment_k_off_kernel__5x_cublas', 'stream': 7, 'count': 12, 'total_duration_us': np.float64(162.43200000000002), 'mean_duration_us': np.float64(13.536000000000001), 'median_duration_us': np.float64(13.488), 'std_dev_duration_us': np.float64(0.16983128883296716), 'min_duration_us': np.float64(13.344), 'max_duration_us': np.float64(13.952)}]</t>
+          <t>[{'name': 'sm90_xmma_gemm_bf16bf16_bf16f32_f32_tn_n_tilesize128x64x64_warpgroupsize1x1x1_execute_segment_k_off_kernel__5x_cublas', 'stream': 7, 'gpu_op_uid': 4124, 'count': 12, 'total_duration_us': np.float64(162.43200000000002), 'mean_duration_us': np.float64(13.536000000000001), 'median_duration_us': np.float64(13.488), 'std_dev_duration_us': np.float64(0.16983128883296716), 'min_duration_us': np.float64(13.344), 'max_duration_us': np.float64(13.952)}]</t>
         </is>
       </c>
       <c r="AM4" t="inlineStr">
@@ -5843,7 +5843,7 @@
       </c>
       <c r="AL5" t="inlineStr">
         <is>
-          <t>[{'name': 'Memset (Device)', 'stream': 7, 'count': 1, 'total_duration_us': np.float64(2.272), 'mean_duration_us': np.float64(2.272), 'median_duration_us': np.float64(2.272), 'std_dev_duration_us': np.float64(0.0), 'min_duration_us': np.float64(2.272), 'max_duration_us': np.float64(2.272)}, {'name': 'void cudnn::engines_precompiled::nchwToNhwcKernel&lt;__nv_bfloat16, __nv_bfloat16, float, false, true, (cudnnKernelDataType_t)0&gt;(cudnn::engines_precompiled::nchw2nhwc_params_t&lt;float&gt;, __nv_bfloat16 const*, __nv_bfloat16*)', 'stream': 7, 'count': 1, 'total_duration_us': np.float64(10.464), 'mean_duration_us': np.float64(10.464), 'median_duration_us': np.float64(10.464), 'std_dev_duration_us': np.float64(0.0), 'min_duration_us': np.float64(10.464), 'max_duration_us': np.float64(10.464)}, {'name': 'Memset (Device)', 'stream': 7, 'count': 1, 'total_duration_us': np.float64(2.112), 'mean_duration_us': np.float64(2.112), 'median_duration_us': np.float64(2.112), 'std_dev_duration_us': np.float64(0.0), 'min_duration_us': np.float64(2.112), 'max_duration_us': np.float64(2.112)}, {'name': 'void cudnn::engines_precompiled::nchwToNhwcKernel&lt;__nv_bfloat16, __nv_bfloat16, float, false, true, (cudnnKernelDataType_t)0&gt;(cudnn::engines_precompiled::nchw2nhwc_params_t&lt;float&gt;, __nv_bfloat16 const*, __nv_bfloat16*)', 'stream': 7, 'count': 1, 'total_duration_us': np.float64(10.4), 'mean_duration_us': np.float64(10.4), 'median_duration_us': np.float64(10.4), 'std_dev_duration_us': np.float64(0.0), 'min_duration_us': np.float64(10.4), 'max_duration_us': np.float64(10.4)}, {'name': 'void cutlass__5x_cudnn::Kernel&lt;cutlass_tensorop_bf16_s16816fprop_optimized_bf16_256x64_32x4_nhwc_align8&gt;(cutlass_tensorop_bf16_s16816fprop_optimized_bf16_256x64_32x4_nhwc_align8::Params)', 'stream': 7, 'count': 1, 'total_duration_us': np.float64(98.176), 'mean_duration_us': np.float64(98.176), 'median_duration_us': np.float64(98.176), 'std_dev_duration_us': np.float64(0.0), 'min_duration_us': np.float64(98.176), 'max_duration_us': np.float64(98.176)}, {'name': 'void cudnn::engines_precompiled::nhwcToNchwKernel&lt;__nv_bfloat16, __nv_bfloat16, float, true, false, (cudnnKernelDataType_t)0&gt;(cudnn::engines_precompiled::nhwc2nchw_params_t&lt;float&gt;, __nv_bfloat16 const*, __nv_bfloat16*)', 'stream': 7, 'count': 1, 'total_duration_us': np.float64(2.208), 'mean_duration_us': np.float64(2.208), 'median_duration_us': np.float64(2.208), 'std_dev_duration_us': np.float64(0.0), 'min_duration_us': np.float64(2.208), 'max_duration_us': np.float64(2.208)}, {'name': 'void at::native::elementwise_kernel&lt;128, 4, at::native::gpu_kernel_impl_nocast&lt;at::native::CUDAFunctor_add&lt;c10::BFloat16&gt; &gt;(at::TensorIteratorBase&amp;, at::native::CUDAFunctor_add&lt;c10::BFloat16&gt; const&amp;)::{lambda(int)#1}&gt;(int, at::native::gpu_kernel_impl_nocast&lt;at::native::CUDAFunctor_add&lt;c10::BFloat16&gt; &gt;(at::TensorIteratorBase&amp;, at::native::CUDAFunctor_add&lt;c10::BFloat16&gt; const&amp;)::{lambda(int)#1})', 'stream': 7, 'count': 1, 'total_duration_us': np.float64(3.968), 'mean_duration_us': np.float64(3.968), 'median_duration_us': np.float64(3.968), 'std_dev_duration_us': np.float64(0.0), 'min_duration_us': np.float64(3.968), 'max_duration_us': np.float64(3.968)}]</t>
+          <t>[{'name': 'Memset (Device)', 'stream': 7, 'gpu_op_uid': 4006, 'count': 1, 'total_duration_us': np.float64(2.272), 'mean_duration_us': np.float64(2.272), 'median_duration_us': np.float64(2.272), 'std_dev_duration_us': np.float64(0.0), 'min_duration_us': np.float64(2.272), 'max_duration_us': np.float64(2.272)}, {'name': 'void cudnn::engines_precompiled::nchwToNhwcKernel&lt;__nv_bfloat16, __nv_bfloat16, float, false, true, (cudnnKernelDataType_t)0&gt;(cudnn::engines_precompiled::nchw2nhwc_params_t&lt;float&gt;, __nv_bfloat16 const*, __nv_bfloat16*)', 'stream': 7, 'gpu_op_uid': 4010, 'count': 1, 'total_duration_us': np.float64(10.464), 'mean_duration_us': np.float64(10.464), 'median_duration_us': np.float64(10.464), 'std_dev_duration_us': np.float64(0.0), 'min_duration_us': np.float64(10.464), 'max_duration_us': np.float64(10.464)}, {'name': 'Memset (Device)', 'stream': 7, 'gpu_op_uid': 4014, 'count': 1, 'total_duration_us': np.float64(2.112), 'mean_duration_us': np.float64(2.112), 'median_duration_us': np.float64(2.112), 'std_dev_duration_us': np.float64(0.0), 'min_duration_us': np.float64(2.112), 'max_duration_us': np.float64(2.112)}, {'name': 'void cudnn::engines_precompiled::nchwToNhwcKernel&lt;__nv_bfloat16, __nv_bfloat16, float, false, true, (cudnnKernelDataType_t)0&gt;(cudnn::engines_precompiled::nchw2nhwc_params_t&lt;float&gt;, __nv_bfloat16 const*, __nv_bfloat16*)', 'stream': 7, 'gpu_op_uid': 4018, 'count': 1, 'total_duration_us': np.float64(10.4), 'mean_duration_us': np.float64(10.4), 'median_duration_us': np.float64(10.4), 'std_dev_duration_us': np.float64(0.0), 'min_duration_us': np.float64(10.4), 'max_duration_us': np.float64(10.4)}, {'name': 'void cutlass__5x_cudnn::Kernel&lt;cutlass_tensorop_bf16_s16816fprop_optimized_bf16_256x64_32x4_nhwc_align8&gt;(cutlass_tensorop_bf16_s16816fprop_optimized_bf16_256x64_32x4_nhwc_align8::Params)', 'stream': 7, 'gpu_op_uid': 4026, 'count': 1, 'total_duration_us': np.float64(98.176), 'mean_duration_us': np.float64(98.176), 'median_duration_us': np.float64(98.176), 'std_dev_duration_us': np.float64(0.0), 'min_duration_us': np.float64(98.176), 'max_duration_us': np.float64(98.176)}, {'name': 'void cudnn::engines_precompiled::nhwcToNchwKernel&lt;__nv_bfloat16, __nv_bfloat16, float, true, false, (cudnnKernelDataType_t)0&gt;(cudnn::engines_precompiled::nhwc2nchw_params_t&lt;float&gt;, __nv_bfloat16 const*, __nv_bfloat16*)', 'stream': 7, 'gpu_op_uid': 4032, 'count': 1, 'total_duration_us': np.float64(2.208), 'mean_duration_us': np.float64(2.208), 'median_duration_us': np.float64(2.208), 'std_dev_duration_us': np.float64(0.0), 'min_duration_us': np.float64(2.208), 'max_duration_us': np.float64(2.208)}, {'name': 'void at::native::elementwise_kernel&lt;128, 4, at::native::gpu_kernel_impl_nocast&lt;at::native::CUDAFunctor_add&lt;c10::BFloat16&gt; &gt;(at::TensorIteratorBase&amp;, at::native::CUDAFunctor_add&lt;c10::BFloat16&gt; const&amp;)::{lambda(int)#1}&gt;(int, at::native::gpu_kernel_impl_nocast&lt;at::native::CUDAFunctor_add&lt;c10::BFloat16&gt; &gt;(at::TensorIteratorBase&amp;, at::native::CUDAFunctor_add&lt;c10::BFloat16&gt; const&amp;)::{lambda(int)#1})', 'stream': 7, 'gpu_op_uid': 4036, 'count': 1, 'total_duration_us': np.float64(3.968), 'mean_duration_us': np.float64(3.968), 'median_duration_us': np.float64(3.968), 'std_dev_duration_us': np.float64(0.0), 'min_duration_us': np.float64(3.968), 'max_duration_us': np.float64(3.968)}]</t>
         </is>
       </c>
       <c r="AM5" t="inlineStr">
@@ -5996,7 +5996,7 @@
       </c>
       <c r="AL6" t="inlineStr">
         <is>
-          <t>[{'name': 'void pytorch_flash::flash_fwd_kernel&lt;pytorch_flash::Flash_fwd_kernel_traits&lt;64, 128, 128, 4, false, false, cutlass::bfloat16_t, pytorch_flash::Flash_kernel_traits&lt;64, 128, 128, 4, cutlass::bfloat16_t&gt; &gt;, false, false, false, false, false, true, false&gt;(pytorch_flash::Flash_fwd_params)', 'stream': 7, 'count': 12, 'total_duration_us': np.float64(122.848), 'mean_duration_us': np.float64(10.237333333333334), 'median_duration_us': np.float64(10.224), 'std_dev_duration_us': np.float64(0.21878045819699932), 'min_duration_us': np.float64(10.016), 'max_duration_us': np.float64(10.848)}]</t>
+          <t>[{'name': 'void pytorch_flash::flash_fwd_kernel&lt;pytorch_flash::Flash_fwd_kernel_traits&lt;64, 128, 128, 4, false, false, cutlass::bfloat16_t, pytorch_flash::Flash_kernel_traits&lt;64, 128, 128, 4, cutlass::bfloat16_t&gt; &gt;, false, false, false, false, false, true, false&gt;(pytorch_flash::Flash_fwd_params)', 'stream': 7, 'gpu_op_uid': 4080, 'count': 12, 'total_duration_us': np.float64(122.848), 'mean_duration_us': np.float64(10.237333333333334), 'median_duration_us': np.float64(10.224), 'std_dev_duration_us': np.float64(0.21878045819699932), 'min_duration_us': np.float64(10.016), 'max_duration_us': np.float64(10.848)}]</t>
         </is>
       </c>
       <c r="AM6" t="inlineStr">
@@ -6153,7 +6153,7 @@
       </c>
       <c r="AL7" t="inlineStr">
         <is>
-          <t>[{'name': 'void at::native::(anonymous namespace)::vectorized_layer_norm_kernel&lt;c10::BFloat16, float&gt;(int, float, c10::BFloat16 const*, c10::BFloat16 const*, c10::BFloat16 const*, float*, float*, c10::BFloat16*)', 'stream': 7, 'count': 25, 'total_duration_us': np.float64(111.20100000000001), 'mean_duration_us': np.float64(4.448040000000001), 'median_duration_us': np.float64(4.448), 'std_dev_duration_us': np.float64(0.10934037863479323), 'min_duration_us': np.float64(4.256), 'max_duration_us': np.float64(4.64)}]</t>
+          <t>[{'name': 'void at::native::(anonymous namespace)::vectorized_layer_norm_kernel&lt;c10::BFloat16, float&gt;(int, float, c10::BFloat16 const*, c10::BFloat16 const*, c10::BFloat16 const*, float*, float*, c10::BFloat16*)', 'stream': 7, 'gpu_op_uid': 4048, 'count': 25, 'total_duration_us': np.float64(111.20100000000001), 'mean_duration_us': np.float64(4.448040000000001), 'median_duration_us': np.float64(4.448), 'std_dev_duration_us': np.float64(0.10934037863479323), 'min_duration_us': np.float64(4.256), 'max_duration_us': np.float64(4.64)}]</t>
         </is>
       </c>
       <c r="AM7" t="inlineStr">
@@ -6280,7 +6280,7 @@
       </c>
       <c r="AL8" t="inlineStr">
         <is>
-          <t>[{'name': 'void at::native::vectorized_elementwise_kernel&lt;4, at::native::GeluCUDAKernelImpl(at::TensorIteratorBase&amp;, at::native::GeluType)::{lambda()#2}::operator()() const::{lambda()#4}::operator()() const::{lambda(c10::BFloat16)#1}, std::array&lt;char*, 2ul&gt; &gt;(int, at::native::GeluCUDAKernelImpl(at::TensorIteratorBase&amp;, at::native::GeluType)::{lambda()#2}::operator()() const::{lambda()#4}::operator()() const::{lambda(c10::BFloat16)#1}, std::array&lt;char*, 2ul&gt;)', 'stream': 7, 'count': 12, 'total_duration_us': np.float64(60.541999999999994), 'mean_duration_us': np.float64(5.045166666666666), 'median_duration_us': np.float64(5.0555), 'std_dev_duration_us': np.float64(0.037739972914080884), 'min_duration_us': np.float64(4.991), 'max_duration_us': np.float64(5.12)}]</t>
+          <t>[{'name': 'void at::native::vectorized_elementwise_kernel&lt;4, at::native::GeluCUDAKernelImpl(at::TensorIteratorBase&amp;, at::native::GeluType)::{lambda()#2}::operator()() const::{lambda()#4}::operator()() const::{lambda(c10::BFloat16)#1}, std::array&lt;char*, 2ul&gt; &gt;(int, at::native::GeluCUDAKernelImpl(at::TensorIteratorBase&amp;, at::native::GeluType)::{lambda()#2}::operator()() const::{lambda()#4}::operator()() const::{lambda(c10::BFloat16)#1}, std::array&lt;char*, 2ul&gt;)', 'stream': 7, 'gpu_op_uid': 4112, 'count': 12, 'total_duration_us': np.float64(60.541999999999994), 'mean_duration_us': np.float64(5.045166666666666), 'median_duration_us': np.float64(5.0555), 'std_dev_duration_us': np.float64(0.037739972914080884), 'min_duration_us': np.float64(4.991), 'max_duration_us': np.float64(5.12)}]</t>
         </is>
       </c>
       <c r="AM8" t="inlineStr">
@@ -6433,7 +6433,7 @@
       </c>
       <c r="AL9" t="inlineStr">
         <is>
-          <t>[{'name': 'void at::native::vectorized_elementwise_kernel&lt;4, at::native::CUDAFunctor_add&lt;c10::BFloat16&gt;, std::array&lt;char*, 3ul&gt; &gt;(int, at::native::CUDAFunctor_add&lt;c10::BFloat16&gt;, std::array&lt;char*, 3ul&gt;)', 'stream': 7, 'count': 24, 'total_duration_us': np.float64(53.536), 'mean_duration_us': np.float64(2.2306666666666666), 'median_duration_us': np.float64(2.2245), 'std_dev_duration_us': np.float64(0.033798011118341686), 'min_duration_us': np.float64(2.176), 'max_duration_us': np.float64(2.304)}]</t>
+          <t>[{'name': 'void at::native::vectorized_elementwise_kernel&lt;4, at::native::CUDAFunctor_add&lt;c10::BFloat16&gt;, std::array&lt;char*, 3ul&gt; &gt;(int, at::native::CUDAFunctor_add&lt;c10::BFloat16&gt;, std::array&lt;char*, 3ul&gt;)', 'stream': 7, 'gpu_op_uid': 4092, 'count': 24, 'total_duration_us': np.float64(53.536), 'mean_duration_us': np.float64(2.2306666666666666), 'median_duration_us': np.float64(2.2245), 'std_dev_duration_us': np.float64(0.033798011118341686), 'min_duration_us': np.float64(2.176), 'max_duration_us': np.float64(2.304)}]</t>
         </is>
       </c>
       <c r="AM9" t="inlineStr">
@@ -6556,7 +6556,7 @@
       </c>
       <c r="AL10" t="inlineStr">
         <is>
-          <t>[{'name': 'void at::native::(anonymous namespace)::CatArrayBatchedCopy&lt;at::native::(anonymous namespace)::OpaqueType&lt;2u&gt;, unsigned int, 3, 64, 64&gt;(at::native::(anonymous namespace)::OpaqueType&lt;2u&gt;*, at::native::(anonymous namespace)::CatArrInputTensorMetadata&lt;at::native::(anonymous namespace)::OpaqueType&lt;2u&gt;, unsigned int, 64, 64&gt;, at::native::(anonymous namespace)::TensorSizeStride&lt;unsigned int, 4u&gt;, int, unsigned int)', 'stream': 7, 'count': 1, 'total_duration_us': np.float64(7.264), 'mean_duration_us': np.float64(7.264), 'median_duration_us': np.float64(7.264), 'std_dev_duration_us': np.float64(0.0), 'min_duration_us': np.float64(7.264), 'max_duration_us': np.float64(7.264)}]</t>
+          <t>[{'name': 'void at::native::(anonymous namespace)::CatArrayBatchedCopy&lt;at::native::(anonymous namespace)::OpaqueType&lt;2u&gt;, unsigned int, 3, 64, 64&gt;(at::native::(anonymous namespace)::OpaqueType&lt;2u&gt;*, at::native::(anonymous namespace)::CatArrInputTensorMetadata&lt;at::native::(anonymous namespace)::OpaqueType&lt;2u&gt;, unsigned int, 64, 64&gt;, at::native::(anonymous namespace)::TensorSizeStride&lt;unsigned int, 4u&gt;, int, unsigned int)', 'stream': 7, 'gpu_op_uid': 4040, 'count': 1, 'total_duration_us': np.float64(7.264), 'mean_duration_us': np.float64(7.264), 'median_duration_us': np.float64(7.264), 'std_dev_duration_us': np.float64(0.0), 'min_duration_us': np.float64(7.264), 'max_duration_us': np.float64(7.264)}]</t>
         </is>
       </c>
       <c r="AM10" t="inlineStr">
@@ -6701,7 +6701,7 @@
       </c>
       <c r="AL11" t="inlineStr">
         <is>
-          <t>[{'name': 'void cutlass::Kernel2&lt;cutlass_80_tensorop_bf16_s16816gemm_relu_bf16_64x64_64x6_tn_align8&gt;(cutlass_80_tensorop_bf16_s16816gemm_relu_bf16_64x64_64x6_tn_align8::Params)', 'stream': 7, 'count': 1, 'total_duration_us': np.float64(6.879), 'mean_duration_us': np.float64(6.879), 'median_duration_us': np.float64(6.879), 'std_dev_duration_us': np.float64(0.0), 'min_duration_us': np.float64(6.879), 'max_duration_us': np.float64(6.879)}]</t>
+          <t>[{'name': 'void cutlass::Kernel2&lt;cutlass_80_tensorop_bf16_s16816gemm_relu_bf16_64x64_64x6_tn_align8&gt;(cutlass_80_tensorop_bf16_s16816gemm_relu_bf16_64x64_64x6_tn_align8::Params)', 'stream': 7, 'gpu_op_uid': 5064, 'count': 1, 'total_duration_us': np.float64(6.879), 'mean_duration_us': np.float64(6.879), 'median_duration_us': np.float64(6.879), 'std_dev_duration_us': np.float64(0.0), 'min_duration_us': np.float64(6.879), 'max_duration_us': np.float64(6.879)}]</t>
         </is>
       </c>
       <c r="AM11" t="inlineStr">
@@ -6850,7 +6850,7 @@
       </c>
       <c r="AL12" t="inlineStr">
         <is>
-          <t>[{'name': 'void at::native::elementwise_kernel&lt;128, 4, at::native::gpu_kernel_impl_nocast&lt;at::native::CUDAFunctor_add&lt;c10::BFloat16&gt; &gt;(at::TensorIteratorBase&amp;, at::native::CUDAFunctor_add&lt;c10::BFloat16&gt; const&amp;)::{lambda(int)#1}&gt;(int, at::native::gpu_kernel_impl_nocast&lt;at::native::CUDAFunctor_add&lt;c10::BFloat16&gt; &gt;(at::TensorIteratorBase&amp;, at::native::CUDAFunctor_add&lt;c10::BFloat16&gt; const&amp;)::{lambda(int)#1})', 'stream': 7, 'count': 1, 'total_duration_us': np.float64(3.777), 'mean_duration_us': np.float64(3.777), 'median_duration_us': np.float64(3.777), 'std_dev_duration_us': np.float64(0.0), 'min_duration_us': np.float64(3.777), 'max_duration_us': np.float64(3.777)}]</t>
+          <t>[{'name': 'void at::native::elementwise_kernel&lt;128, 4, at::native::gpu_kernel_impl_nocast&lt;at::native::CUDAFunctor_add&lt;c10::BFloat16&gt; &gt;(at::TensorIteratorBase&amp;, at::native::CUDAFunctor_add&lt;c10::BFloat16&gt; const&amp;)::{lambda(int)#1}&gt;(int, at::native::gpu_kernel_impl_nocast&lt;at::native::CUDAFunctor_add&lt;c10::BFloat16&gt; &gt;(at::TensorIteratorBase&amp;, at::native::CUDAFunctor_add&lt;c10::BFloat16&gt; const&amp;)::{lambda(int)#1})', 'stream': 7, 'gpu_op_uid': 4044, 'count': 1, 'total_duration_us': np.float64(3.777), 'mean_duration_us': np.float64(3.777), 'median_duration_us': np.float64(3.777), 'std_dev_duration_us': np.float64(0.0), 'min_duration_us': np.float64(3.777), 'max_duration_us': np.float64(3.777)}]</t>
         </is>
       </c>
       <c r="AM12" t="inlineStr">
@@ -6973,7 +6973,7 @@
       </c>
       <c r="AL13" t="inlineStr">
         <is>
-          <t>[{'name': 'void at::native::vectorized_elementwise_kernel&lt;4, at::native::tanh_kernel_cuda(at::TensorIteratorBase&amp;)::{lambda()#2}::operator()() const::{lambda()#4}::operator()() const::{lambda(c10::BFloat16)#1}, std::array&lt;char*, 2ul&gt; &gt;(int, at::native::tanh_kernel_cuda(at::TensorIteratorBase&amp;)::{lambda()#2}::operator()() const::{lambda()#4}::operator()() const::{lambda(c10::BFloat16)#1}, std::array&lt;char*, 2ul&gt;)', 'stream': 7, 'count': 1, 'total_duration_us': np.float64(1.505), 'mean_duration_us': np.float64(1.505), 'median_duration_us': np.float64(1.505), 'std_dev_duration_us': np.float64(0.0), 'min_duration_us': np.float64(1.505), 'max_duration_us': np.float64(1.505)}]</t>
+          <t>[{'name': 'void at::native::vectorized_elementwise_kernel&lt;4, at::native::tanh_kernel_cuda(at::TensorIteratorBase&amp;)::{lambda()#2}::operator()() const::{lambda()#4}::operator()() const::{lambda(c10::BFloat16)#1}, std::array&lt;char*, 2ul&gt; &gt;(int, at::native::tanh_kernel_cuda(at::TensorIteratorBase&amp;)::{lambda()#2}::operator()() const::{lambda()#4}::operator()() const::{lambda(c10::BFloat16)#1}, std::array&lt;char*, 2ul&gt;)', 'stream': 7, 'gpu_op_uid': 5068, 'count': 1, 'total_duration_us': np.float64(1.505), 'mean_duration_us': np.float64(1.505), 'median_duration_us': np.float64(1.505), 'std_dev_duration_us': np.float64(0.0), 'min_duration_us': np.float64(1.505), 'max_duration_us': np.float64(1.505)}]</t>
         </is>
       </c>
       <c r="AM13" t="inlineStr">
@@ -7315,7 +7315,7 @@
       </c>
       <c r="AA2" t="inlineStr">
         <is>
-          <t>[{'name': 'void cutlass::Kernel2&lt;cutlass_80_tensorop_bf16_s16816gemm_relu_bf16_128x64_64x6_tn_align8&gt;(cutlass_80_tensorop_bf16_s16816gemm_relu_bf16_128x64_64x6_tn_align8::Params)', 'stream': 7, 'count': 48, 'total_duration_us': np.float64(399.136), 'mean_duration_us': np.float64(8.315333333333333), 'median_duration_us': np.float64(8.256), 'std_dev_duration_us': np.float64(0.13305517861231703), 'min_duration_us': np.float64(8.128), 'max_duration_us': np.float64(8.64)}]</t>
+          <t>[{'name': 'void cutlass::Kernel2&lt;cutlass_80_tensorop_bf16_s16816gemm_relu_bf16_128x64_64x6_tn_align8&gt;(cutlass_80_tensorop_bf16_s16816gemm_relu_bf16_128x64_64x6_tn_align8::Params)', 'stream': 7, 'gpu_op_uid': 4056, 'count': 48, 'total_duration_us': np.float64(399.136), 'mean_duration_us': np.float64(8.315333333333333), 'median_duration_us': np.float64(8.256), 'std_dev_duration_us': np.float64(0.13305517861231703), 'min_duration_us': np.float64(8.128), 'max_duration_us': np.float64(8.64)}]</t>
         </is>
       </c>
       <c r="AB2" t="inlineStr">
@@ -7475,7 +7475,7 @@
       </c>
       <c r="AA3" t="inlineStr">
         <is>
-          <t>[{'name': 'sm90_xmma_gemm_bf16bf16_bf16f32_f32_tn_n_tilesize128x128x64_warpgroupsize1x1x1_execute_segment_k_off_kernel__5x_cublas', 'stream': 7, 'count': 12, 'total_duration_us': np.float64(166.59), 'mean_duration_us': np.float64(13.8825), 'median_duration_us': np.float64(13.8875), 'std_dev_duration_us': np.float64(0.10183278777813505), 'min_duration_us': np.float64(13.76), 'max_duration_us': np.float64(14.176)}]</t>
+          <t>[{'name': 'sm90_xmma_gemm_bf16bf16_bf16f32_f32_tn_n_tilesize128x128x64_warpgroupsize1x1x1_execute_segment_k_off_kernel__5x_cublas', 'stream': 7, 'gpu_op_uid': 4108, 'count': 12, 'total_duration_us': np.float64(166.59), 'mean_duration_us': np.float64(13.8825), 'median_duration_us': np.float64(13.8875), 'std_dev_duration_us': np.float64(0.10183278777813505), 'min_duration_us': np.float64(13.76), 'max_duration_us': np.float64(14.176)}]</t>
         </is>
       </c>
       <c r="AB3" t="inlineStr">
@@ -7635,7 +7635,7 @@
       </c>
       <c r="AA4" t="inlineStr">
         <is>
-          <t>[{'name': 'sm90_xmma_gemm_bf16bf16_bf16f32_f32_tn_n_tilesize128x64x64_warpgroupsize1x1x1_execute_segment_k_off_kernel__5x_cublas', 'stream': 7, 'count': 12, 'total_duration_us': np.float64(162.43200000000002), 'mean_duration_us': np.float64(13.536000000000001), 'median_duration_us': np.float64(13.488), 'std_dev_duration_us': np.float64(0.16983128883296716), 'min_duration_us': np.float64(13.344), 'max_duration_us': np.float64(13.952)}]</t>
+          <t>[{'name': 'sm90_xmma_gemm_bf16bf16_bf16f32_f32_tn_n_tilesize128x64x64_warpgroupsize1x1x1_execute_segment_k_off_kernel__5x_cublas', 'stream': 7, 'gpu_op_uid': 4124, 'count': 12, 'total_duration_us': np.float64(162.43200000000002), 'mean_duration_us': np.float64(13.536000000000001), 'median_duration_us': np.float64(13.488), 'std_dev_duration_us': np.float64(0.16983128883296716), 'min_duration_us': np.float64(13.344), 'max_duration_us': np.float64(13.952)}]</t>
         </is>
       </c>
       <c r="AB4" t="inlineStr">
@@ -7791,7 +7791,7 @@
       </c>
       <c r="AA5" t="inlineStr">
         <is>
-          <t>[{'name': 'void cutlass::Kernel2&lt;cutlass_80_tensorop_bf16_s16816gemm_relu_bf16_64x64_64x6_tn_align8&gt;(cutlass_80_tensorop_bf16_s16816gemm_relu_bf16_64x64_64x6_tn_align8::Params)', 'stream': 7, 'count': 1, 'total_duration_us': np.float64(6.879), 'mean_duration_us': np.float64(6.879), 'median_duration_us': np.float64(6.879), 'std_dev_duration_us': np.float64(0.0), 'min_duration_us': np.float64(6.879), 'max_duration_us': np.float64(6.879)}]</t>
+          <t>[{'name': 'void cutlass::Kernel2&lt;cutlass_80_tensorop_bf16_s16816gemm_relu_bf16_64x64_64x6_tn_align8&gt;(cutlass_80_tensorop_bf16_s16816gemm_relu_bf16_64x64_64x6_tn_align8::Params)', 'stream': 7, 'gpu_op_uid': 5064, 'count': 1, 'total_duration_us': np.float64(6.879), 'mean_duration_us': np.float64(6.879), 'median_duration_us': np.float64(6.879), 'std_dev_duration_us': np.float64(0.0), 'min_duration_us': np.float64(6.879), 'max_duration_us': np.float64(6.879)}]</t>
         </is>
       </c>
       <c r="AB5" t="inlineStr">
@@ -8181,7 +8181,7 @@
       <c r="AB2" t="inlineStr"/>
       <c r="AC2" t="inlineStr">
         <is>
-          <t>[{'name': 'void pytorch_flash::flash_fwd_kernel&lt;pytorch_flash::Flash_fwd_kernel_traits&lt;64, 128, 128, 4, false, false, cutlass::bfloat16_t, pytorch_flash::Flash_kernel_traits&lt;64, 128, 128, 4, cutlass::bfloat16_t&gt; &gt;, false, false, false, false, false, true, false&gt;(pytorch_flash::Flash_fwd_params)', 'stream': 7, 'count': 12, 'total_duration_us': np.float64(122.848), 'mean_duration_us': np.float64(10.237333333333334), 'median_duration_us': np.float64(10.224), 'std_dev_duration_us': np.float64(0.21878045819699932), 'min_duration_us': np.float64(10.016), 'max_duration_us': np.float64(10.848)}]</t>
+          <t>[{'name': 'void pytorch_flash::flash_fwd_kernel&lt;pytorch_flash::Flash_fwd_kernel_traits&lt;64, 128, 128, 4, false, false, cutlass::bfloat16_t, pytorch_flash::Flash_kernel_traits&lt;64, 128, 128, 4, cutlass::bfloat16_t&gt; &gt;, false, false, false, false, false, true, false&gt;(pytorch_flash::Flash_fwd_params)', 'stream': 7, 'gpu_op_uid': 4080, 'count': 12, 'total_duration_us': np.float64(122.848), 'mean_duration_us': np.float64(10.237333333333334), 'median_duration_us': np.float64(10.224), 'std_dev_duration_us': np.float64(0.21878045819699932), 'min_duration_us': np.float64(10.016), 'max_duration_us': np.float64(10.848)}]</t>
         </is>
       </c>
       <c r="AD2" t="inlineStr">
@@ -8603,7 +8603,7 @@
       </c>
       <c r="AF2" t="inlineStr">
         <is>
-          <t>[{'name': 'Memset (Device)', 'stream': 7, 'count': 1, 'total_duration_us': np.float64(2.272), 'mean_duration_us': np.float64(2.272), 'median_duration_us': np.float64(2.272), 'std_dev_duration_us': np.float64(0.0), 'min_duration_us': np.float64(2.272), 'max_duration_us': np.float64(2.272)}, {'name': 'void cudnn::engines_precompiled::nchwToNhwcKernel&lt;__nv_bfloat16, __nv_bfloat16, float, false, true, (cudnnKernelDataType_t)0&gt;(cudnn::engines_precompiled::nchw2nhwc_params_t&lt;float&gt;, __nv_bfloat16 const*, __nv_bfloat16*)', 'stream': 7, 'count': 1, 'total_duration_us': np.float64(10.464), 'mean_duration_us': np.float64(10.464), 'median_duration_us': np.float64(10.464), 'std_dev_duration_us': np.float64(0.0), 'min_duration_us': np.float64(10.464), 'max_duration_us': np.float64(10.464)}, {'name': 'Memset (Device)', 'stream': 7, 'count': 1, 'total_duration_us': np.float64(2.112), 'mean_duration_us': np.float64(2.112), 'median_duration_us': np.float64(2.112), 'std_dev_duration_us': np.float64(0.0), 'min_duration_us': np.float64(2.112), 'max_duration_us': np.float64(2.112)}, {'name': 'void cudnn::engines_precompiled::nchwToNhwcKernel&lt;__nv_bfloat16, __nv_bfloat16, float, false, true, (cudnnKernelDataType_t)0&gt;(cudnn::engines_precompiled::nchw2nhwc_params_t&lt;float&gt;, __nv_bfloat16 const*, __nv_bfloat16*)', 'stream': 7, 'count': 1, 'total_duration_us': np.float64(10.4), 'mean_duration_us': np.float64(10.4), 'median_duration_us': np.float64(10.4), 'std_dev_duration_us': np.float64(0.0), 'min_duration_us': np.float64(10.4), 'max_duration_us': np.float64(10.4)}, {'name': 'void cutlass__5x_cudnn::Kernel&lt;cutlass_tensorop_bf16_s16816fprop_optimized_bf16_256x64_32x4_nhwc_align8&gt;(cutlass_tensorop_bf16_s16816fprop_optimized_bf16_256x64_32x4_nhwc_align8::Params)', 'stream': 7, 'count': 1, 'total_duration_us': np.float64(98.176), 'mean_duration_us': np.float64(98.176), 'median_duration_us': np.float64(98.176), 'std_dev_duration_us': np.float64(0.0), 'min_duration_us': np.float64(98.176), 'max_duration_us': np.float64(98.176)}, {'name': 'void cudnn::engines_precompiled::nhwcToNchwKernel&lt;__nv_bfloat16, __nv_bfloat16, float, true, false, (cudnnKernelDataType_t)0&gt;(cudnn::engines_precompiled::nhwc2nchw_params_t&lt;float&gt;, __nv_bfloat16 const*, __nv_bfloat16*)', 'stream': 7, 'count': 1, 'total_duration_us': np.float64(2.208), 'mean_duration_us': np.float64(2.208), 'median_duration_us': np.float64(2.208), 'std_dev_duration_us': np.float64(0.0), 'min_duration_us': np.float64(2.208), 'max_duration_us': np.float64(2.208)}, {'name': 'void at::native::elementwise_kernel&lt;128, 4, at::native::gpu_kernel_impl_nocast&lt;at::native::CUDAFunctor_add&lt;c10::BFloat16&gt; &gt;(at::TensorIteratorBase&amp;, at::native::CUDAFunctor_add&lt;c10::BFloat16&gt; const&amp;)::{lambda(int)#1}&gt;(int, at::native::gpu_kernel_impl_nocast&lt;at::native::CUDAFunctor_add&lt;c10::BFloat16&gt; &gt;(at::TensorIteratorBase&amp;, at::native::CUDAFunctor_add&lt;c10::BFloat16&gt; const&amp;)::{lambda(int)#1})', 'stream': 7, 'count': 1, 'total_duration_us': np.float64(3.968), 'mean_duration_us': np.float64(3.968), 'median_duration_us': np.float64(3.968), 'std_dev_duration_us': np.float64(0.0), 'min_duration_us': np.float64(3.968), 'max_duration_us': np.float64(3.968)}]</t>
+          <t>[{'name': 'Memset (Device)', 'stream': 7, 'gpu_op_uid': 4006, 'count': 1, 'total_duration_us': np.float64(2.272), 'mean_duration_us': np.float64(2.272), 'median_duration_us': np.float64(2.272), 'std_dev_duration_us': np.float64(0.0), 'min_duration_us': np.float64(2.272), 'max_duration_us': np.float64(2.272)}, {'name': 'void cudnn::engines_precompiled::nchwToNhwcKernel&lt;__nv_bfloat16, __nv_bfloat16, float, false, true, (cudnnKernelDataType_t)0&gt;(cudnn::engines_precompiled::nchw2nhwc_params_t&lt;float&gt;, __nv_bfloat16 const*, __nv_bfloat16*)', 'stream': 7, 'gpu_op_uid': 4010, 'count': 1, 'total_duration_us': np.float64(10.464), 'mean_duration_us': np.float64(10.464), 'median_duration_us': np.float64(10.464), 'std_dev_duration_us': np.float64(0.0), 'min_duration_us': np.float64(10.464), 'max_duration_us': np.float64(10.464)}, {'name': 'Memset (Device)', 'stream': 7, 'gpu_op_uid': 4014, 'count': 1, 'total_duration_us': np.float64(2.112), 'mean_duration_us': np.float64(2.112), 'median_duration_us': np.float64(2.112), 'std_dev_duration_us': np.float64(0.0), 'min_duration_us': np.float64(2.112), 'max_duration_us': np.float64(2.112)}, {'name': 'void cudnn::engines_precompiled::nchwToNhwcKernel&lt;__nv_bfloat16, __nv_bfloat16, float, false, true, (cudnnKernelDataType_t)0&gt;(cudnn::engines_precompiled::nchw2nhwc_params_t&lt;float&gt;, __nv_bfloat16 const*, __nv_bfloat16*)', 'stream': 7, 'gpu_op_uid': 4018, 'count': 1, 'total_duration_us': np.float64(10.4), 'mean_duration_us': np.float64(10.4), 'median_duration_us': np.float64(10.4), 'std_dev_duration_us': np.float64(0.0), 'min_duration_us': np.float64(10.4), 'max_duration_us': np.float64(10.4)}, {'name': 'void cutlass__5x_cudnn::Kernel&lt;cutlass_tensorop_bf16_s16816fprop_optimized_bf16_256x64_32x4_nhwc_align8&gt;(cutlass_tensorop_bf16_s16816fprop_optimized_bf16_256x64_32x4_nhwc_align8::Params)', 'stream': 7, 'gpu_op_uid': 4026, 'count': 1, 'total_duration_us': np.float64(98.176), 'mean_duration_us': np.float64(98.176), 'median_duration_us': np.float64(98.176), 'std_dev_duration_us': np.float64(0.0), 'min_duration_us': np.float64(98.176), 'max_duration_us': np.float64(98.176)}, {'name': 'void cudnn::engines_precompiled::nhwcToNchwKernel&lt;__nv_bfloat16, __nv_bfloat16, float, true, false, (cudnnKernelDataType_t)0&gt;(cudnn::engines_precompiled::nhwc2nchw_params_t&lt;float&gt;, __nv_bfloat16 const*, __nv_bfloat16*)', 'stream': 7, 'gpu_op_uid': 4032, 'count': 1, 'total_duration_us': np.float64(2.208), 'mean_duration_us': np.float64(2.208), 'median_duration_us': np.float64(2.208), 'std_dev_duration_us': np.float64(0.0), 'min_duration_us': np.float64(2.208), 'max_duration_us': np.float64(2.208)}, {'name': 'void at::native::elementwise_kernel&lt;128, 4, at::native::gpu_kernel_impl_nocast&lt;at::native::CUDAFunctor_add&lt;c10::BFloat16&gt; &gt;(at::TensorIteratorBase&amp;, at::native::CUDAFunctor_add&lt;c10::BFloat16&gt; const&amp;)::{lambda(int)#1}&gt;(int, at::native::gpu_kernel_impl_nocast&lt;at::native::CUDAFunctor_add&lt;c10::BFloat16&gt; &gt;(at::TensorIteratorBase&amp;, at::native::CUDAFunctor_add&lt;c10::BFloat16&gt; const&amp;)::{lambda(int)#1})', 'stream': 7, 'gpu_op_uid': 4036, 'count': 1, 'total_duration_us': np.float64(3.968), 'mean_duration_us': np.float64(3.968), 'median_duration_us': np.float64(3.968), 'std_dev_duration_us': np.float64(0.0), 'min_duration_us': np.float64(3.968), 'max_duration_us': np.float64(3.968)}]</t>
         </is>
       </c>
       <c r="AG2" t="inlineStr">
@@ -8953,7 +8953,7 @@
       </c>
       <c r="Y2" t="inlineStr">
         <is>
-          <t>[{'name': 'void at::native::vectorized_elementwise_kernel&lt;4, at::native::CUDAFunctor_add&lt;c10::BFloat16&gt;, std::array&lt;char*, 3ul&gt; &gt;(int, at::native::CUDAFunctor_add&lt;c10::BFloat16&gt;, std::array&lt;char*, 3ul&gt;)', 'stream': 7, 'count': 24, 'total_duration_us': np.float64(53.536), 'mean_duration_us': np.float64(2.2306666666666666), 'median_duration_us': np.float64(2.2245), 'std_dev_duration_us': np.float64(0.033798011118341686), 'min_duration_us': np.float64(2.176), 'max_duration_us': np.float64(2.304)}]</t>
+          <t>[{'name': 'void at::native::vectorized_elementwise_kernel&lt;4, at::native::CUDAFunctor_add&lt;c10::BFloat16&gt;, std::array&lt;char*, 3ul&gt; &gt;(int, at::native::CUDAFunctor_add&lt;c10::BFloat16&gt;, std::array&lt;char*, 3ul&gt;)', 'stream': 7, 'gpu_op_uid': 4092, 'count': 24, 'total_duration_us': np.float64(53.536), 'mean_duration_us': np.float64(2.2306666666666666), 'median_duration_us': np.float64(2.2245), 'std_dev_duration_us': np.float64(0.033798011118341686), 'min_duration_us': np.float64(2.176), 'max_duration_us': np.float64(2.304)}]</t>
         </is>
       </c>
       <c r="Z2" t="inlineStr">
@@ -9095,7 +9095,7 @@
       </c>
       <c r="Y3" t="inlineStr">
         <is>
-          <t>[{'name': 'void at::native::elementwise_kernel&lt;128, 4, at::native::gpu_kernel_impl_nocast&lt;at::native::CUDAFunctor_add&lt;c10::BFloat16&gt; &gt;(at::TensorIteratorBase&amp;, at::native::CUDAFunctor_add&lt;c10::BFloat16&gt; const&amp;)::{lambda(int)#1}&gt;(int, at::native::gpu_kernel_impl_nocast&lt;at::native::CUDAFunctor_add&lt;c10::BFloat16&gt; &gt;(at::TensorIteratorBase&amp;, at::native::CUDAFunctor_add&lt;c10::BFloat16&gt; const&amp;)::{lambda(int)#1})', 'stream': 7, 'count': 1, 'total_duration_us': np.float64(3.968), 'mean_duration_us': np.float64(3.968), 'median_duration_us': np.float64(3.968), 'std_dev_duration_us': np.float64(0.0), 'min_duration_us': np.float64(3.968), 'max_duration_us': np.float64(3.968)}]</t>
+          <t>[{'name': 'void at::native::elementwise_kernel&lt;128, 4, at::native::gpu_kernel_impl_nocast&lt;at::native::CUDAFunctor_add&lt;c10::BFloat16&gt; &gt;(at::TensorIteratorBase&amp;, at::native::CUDAFunctor_add&lt;c10::BFloat16&gt; const&amp;)::{lambda(int)#1}&gt;(int, at::native::gpu_kernel_impl_nocast&lt;at::native::CUDAFunctor_add&lt;c10::BFloat16&gt; &gt;(at::TensorIteratorBase&amp;, at::native::CUDAFunctor_add&lt;c10::BFloat16&gt; const&amp;)::{lambda(int)#1})', 'stream': 7, 'gpu_op_uid': 4036, 'count': 1, 'total_duration_us': np.float64(3.968), 'mean_duration_us': np.float64(3.968), 'median_duration_us': np.float64(3.968), 'std_dev_duration_us': np.float64(0.0), 'min_duration_us': np.float64(3.968), 'max_duration_us': np.float64(3.968)}]</t>
         </is>
       </c>
       <c r="Z3" t="inlineStr">
@@ -9235,7 +9235,7 @@
       </c>
       <c r="Y4" t="inlineStr">
         <is>
-          <t>[{'name': 'void at::native::elementwise_kernel&lt;128, 4, at::native::gpu_kernel_impl_nocast&lt;at::native::CUDAFunctor_add&lt;c10::BFloat16&gt; &gt;(at::TensorIteratorBase&amp;, at::native::CUDAFunctor_add&lt;c10::BFloat16&gt; const&amp;)::{lambda(int)#1}&gt;(int, at::native::gpu_kernel_impl_nocast&lt;at::native::CUDAFunctor_add&lt;c10::BFloat16&gt; &gt;(at::TensorIteratorBase&amp;, at::native::CUDAFunctor_add&lt;c10::BFloat16&gt; const&amp;)::{lambda(int)#1})', 'stream': 7, 'count': 1, 'total_duration_us': np.float64(3.777), 'mean_duration_us': np.float64(3.777), 'median_duration_us': np.float64(3.777), 'std_dev_duration_us': np.float64(0.0), 'min_duration_us': np.float64(3.777), 'max_duration_us': np.float64(3.777)}]</t>
+          <t>[{'name': 'void at::native::elementwise_kernel&lt;128, 4, at::native::gpu_kernel_impl_nocast&lt;at::native::CUDAFunctor_add&lt;c10::BFloat16&gt; &gt;(at::TensorIteratorBase&amp;, at::native::CUDAFunctor_add&lt;c10::BFloat16&gt; const&amp;)::{lambda(int)#1}&gt;(int, at::native::gpu_kernel_impl_nocast&lt;at::native::CUDAFunctor_add&lt;c10::BFloat16&gt; &gt;(at::TensorIteratorBase&amp;, at::native::CUDAFunctor_add&lt;c10::BFloat16&gt; const&amp;)::{lambda(int)#1})', 'stream': 7, 'gpu_op_uid': 4044, 'count': 1, 'total_duration_us': np.float64(3.777), 'mean_duration_us': np.float64(3.777), 'median_duration_us': np.float64(3.777), 'std_dev_duration_us': np.float64(0.0), 'min_duration_us': np.float64(3.777), 'max_duration_us': np.float64(3.777)}]</t>
         </is>
       </c>
       <c r="Z4" t="inlineStr">

</xml_diff>